<commit_message>
change in Day 5 material
</commit_message>
<xml_diff>
--- a/Day 3/Datasets/PCA_FA_Factor_Analysis_Survey.xlsx
+++ b/Day 3/Datasets/PCA_FA_Factor_Analysis_Survey.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Academics\MDPs\5-Day Online Hands-on Workshop (MDP) on AIML\Day 3\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08356AC8-A6D8-4F9A-A6DA-CE4B05F3C061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22895761-BCAD-4902-8FDA-B8F162C0258A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
   <si>
     <t>age</t>
   </si>
@@ -445,19 +446,19 @@
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <f ca="1">RANDBETWEEN(20, 80)</f>
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="B2">
         <f ca="1">RANDBETWEEN(20, 80)</f>
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2">
         <f ca="1">RANDBETWEEN(1, 3)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <f ca="1">RANDBETWEEN(1, 3)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <f ca="1">RANDBETWEEN(1, 2)</f>
@@ -465,11 +466,11 @@
       </c>
       <c r="F2">
         <f ca="1">RANDBETWEEN(1, 5)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <f t="shared" ref="G2:N2" ca="1" si="0">RANDBETWEEN(1, 5)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H2">
         <f t="shared" ca="1" si="0"/>
@@ -477,19 +478,19 @@
       </c>
       <c r="I2">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K2">
         <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L2">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
         <f t="shared" ca="1" si="0"/>
@@ -497,21 +498,21 @@
       </c>
       <c r="N2">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" ref="A3:B31" ca="1" si="1">RANDBETWEEN(20, 80)</f>
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B3">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C3">
         <f t="shared" ref="C3:D31" ca="1" si="2">RANDBETWEEN(1, 3)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
         <f t="shared" ca="1" si="2"/>
@@ -527,11 +528,11 @@
       </c>
       <c r="G3">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I3">
         <f t="shared" ca="1" si="4"/>
@@ -539,7 +540,7 @@
       </c>
       <c r="J3">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K3">
         <f t="shared" ca="1" si="4"/>
@@ -547,41 +548,41 @@
       </c>
       <c r="L3">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M3">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N3">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C4">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4">
         <f t="shared" ca="1" si="4"/>
@@ -589,27 +590,27 @@
       </c>
       <c r="H4">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M4">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4">
         <f t="shared" ca="1" si="4"/>
@@ -619,15 +620,15 @@
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" ca="1" si="1"/>
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <f t="shared" ca="1" si="1"/>
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5">
         <f t="shared" ca="1" si="2"/>
@@ -639,11 +640,11 @@
       </c>
       <c r="F5">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <f t="shared" ca="1" si="4"/>
@@ -651,45 +652,45 @@
       </c>
       <c r="I5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L5">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N5">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="B6">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="C6">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6">
         <f t="shared" ca="1" si="3"/>
@@ -697,15 +698,15 @@
       </c>
       <c r="F6">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G6">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6">
         <f t="shared" ca="1" si="4"/>
@@ -713,11 +714,11 @@
       </c>
       <c r="J6">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6">
         <f t="shared" ca="1" si="4"/>
@@ -725,33 +726,33 @@
       </c>
       <c r="M6">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N6">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="B7">
         <f t="shared" ca="1" si="1"/>
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="C7">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7">
         <f t="shared" ca="1" si="4"/>
@@ -759,69 +760,69 @@
       </c>
       <c r="G7">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J7">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M7">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B8">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G8">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H8">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8">
         <f t="shared" ca="1" si="4"/>
@@ -829,11 +830,11 @@
       </c>
       <c r="J8">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L8">
         <f t="shared" ca="1" si="4"/>
@@ -845,41 +846,41 @@
       </c>
       <c r="N8">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" ca="1" si="1"/>
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B9">
         <f t="shared" ca="1" si="1"/>
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C9">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H9">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I9">
         <f t="shared" ca="1" si="4"/>
@@ -887,7 +888,7 @@
       </c>
       <c r="J9">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9">
         <f t="shared" ca="1" si="4"/>
@@ -895,29 +896,29 @@
       </c>
       <c r="L9">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M9">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="B10">
         <f t="shared" ca="1" si="1"/>
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="C10">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="2"/>
@@ -929,7 +930,7 @@
       </c>
       <c r="F10">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="4"/>
@@ -937,49 +938,49 @@
       </c>
       <c r="H10">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M10">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B11">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="C11">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <f t="shared" ca="1" si="3"/>
@@ -987,11 +988,11 @@
       </c>
       <c r="F11">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H11">
         <f t="shared" ca="1" si="4"/>
@@ -999,65 +1000,65 @@
       </c>
       <c r="I11">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J11">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K11">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M11">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N11">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B12">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="C12">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G12">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I12">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12">
         <f t="shared" ca="1" si="4"/>
@@ -1069,25 +1070,25 @@
       </c>
       <c r="L12">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" ca="1" si="1"/>
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="B13">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C13">
         <f t="shared" ca="1" si="2"/>
@@ -1095,7 +1096,7 @@
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13">
         <f t="shared" ca="1" si="3"/>
@@ -1103,15 +1104,15 @@
       </c>
       <c r="F13">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I13">
         <f t="shared" ca="1" si="4"/>
@@ -1119,33 +1120,33 @@
       </c>
       <c r="J13">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K13">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L13">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M13">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N13">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="B14">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C14">
         <f t="shared" ca="1" si="2"/>
@@ -1161,61 +1162,61 @@
       </c>
       <c r="F14">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G14">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I14">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L14">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N14">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B15">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="C15">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15">
         <f t="shared" ca="1" si="4"/>
@@ -1227,41 +1228,41 @@
       </c>
       <c r="H15">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I15">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J15">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K15">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L15">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M15">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N15">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="B16">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C16">
         <f t="shared" ca="1" si="2"/>
@@ -1269,31 +1270,31 @@
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I16">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K16">
         <f t="shared" ca="1" si="4"/>
@@ -1301,7 +1302,7 @@
       </c>
       <c r="L16">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M16">
         <f t="shared" ca="1" si="4"/>
@@ -1309,13 +1310,13 @@
       </c>
       <c r="N16">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <f t="shared" ca="1" si="1"/>
@@ -1327,19 +1328,19 @@
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17">
         <f t="shared" ca="1" si="4"/>
@@ -1347,7 +1348,7 @@
       </c>
       <c r="I17">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J17">
         <f t="shared" ca="1" si="4"/>
@@ -1359,33 +1360,33 @@
       </c>
       <c r="L17">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M17">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N17">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B18">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="C18">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18">
         <f t="shared" ca="1" si="3"/>
@@ -1393,19 +1394,19 @@
       </c>
       <c r="F18">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I18">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <f t="shared" ca="1" si="4"/>
@@ -1417,21 +1418,21 @@
       </c>
       <c r="L18">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M18">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N18">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="B19">
         <f t="shared" ca="1" si="1"/>
@@ -1439,7 +1440,7 @@
       </c>
       <c r="C19">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19">
         <f t="shared" ca="1" si="2"/>
@@ -1447,15 +1448,15 @@
       </c>
       <c r="E19">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G19">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H19">
         <f t="shared" ca="1" si="4"/>
@@ -1463,7 +1464,7 @@
       </c>
       <c r="I19">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J19">
         <f t="shared" ca="1" si="4"/>
@@ -1471,11 +1472,11 @@
       </c>
       <c r="K19">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L19">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M19">
         <f t="shared" ca="1" si="4"/>
@@ -1489,15 +1490,15 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B20">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="C20">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="2"/>
@@ -1505,19 +1506,19 @@
       </c>
       <c r="E20">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H20">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I20">
         <f t="shared" ca="1" si="4"/>
@@ -1525,19 +1526,19 @@
       </c>
       <c r="J20">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K20">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L20">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N20">
         <f t="shared" ca="1" si="4"/>
@@ -1547,23 +1548,23 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B21">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C21">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21">
         <f t="shared" ca="1" si="4"/>
@@ -1571,23 +1572,23 @@
       </c>
       <c r="G21">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H21">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <f t="shared" ca="1" si="4"/>
@@ -1605,31 +1606,31 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" ca="1" si="1"/>
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B22">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C22">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G22">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H22">
         <f t="shared" ca="1" si="4"/>
@@ -1637,11 +1638,11 @@
       </c>
       <c r="I22">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J22">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22">
         <f t="shared" ca="1" si="4"/>
@@ -1649,7 +1650,7 @@
       </c>
       <c r="L22">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M22">
         <f t="shared" ca="1" si="4"/>
@@ -1657,25 +1658,25 @@
       </c>
       <c r="N22">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" ca="1" si="1"/>
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B23">
         <f t="shared" ca="1" si="1"/>
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="C23">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23">
         <f t="shared" ca="1" si="3"/>
@@ -1683,31 +1684,31 @@
       </c>
       <c r="F23">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H23">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J23">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K23">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L23">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M23">
         <f t="shared" ca="1" si="4"/>
@@ -1721,15 +1722,15 @@
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" ca="1" si="1"/>
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B24">
         <f t="shared" ca="1" si="1"/>
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="C24">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24">
         <f t="shared" ca="1" si="2"/>
@@ -1737,7 +1738,7 @@
       </c>
       <c r="E24">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24">
         <f t="shared" ca="1" si="4"/>
@@ -1745,123 +1746,123 @@
       </c>
       <c r="G24">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H24">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I24">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J24">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K24">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L24">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M24">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N24">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" ca="1" si="1"/>
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="B25">
         <f t="shared" ca="1" si="1"/>
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="C25">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G25">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I25">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L25">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M25">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N25">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" ca="1" si="1"/>
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="C26">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G26">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H26">
         <f t="shared" ca="1" si="4"/>
@@ -1869,41 +1870,41 @@
       </c>
       <c r="I26">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J26">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K26">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L26">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M26">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N26">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C27">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27">
         <f t="shared" ca="1" si="2"/>
@@ -1915,7 +1916,7 @@
       </c>
       <c r="F27">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27">
         <f t="shared" ca="1" si="4"/>
@@ -1939,21 +1940,21 @@
       </c>
       <c r="L27">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M27">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N27">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="B28">
         <f t="shared" ca="1" si="1"/>
@@ -1977,7 +1978,7 @@
       </c>
       <c r="G28">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28">
         <f t="shared" ca="1" si="4"/>
@@ -1985,11 +1986,11 @@
       </c>
       <c r="I28">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J28">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K28">
         <f t="shared" ca="1" si="4"/>
@@ -1997,25 +1998,25 @@
       </c>
       <c r="L28">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M28">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" ca="1" si="1"/>
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="B29">
         <f t="shared" ca="1" si="1"/>
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C29">
         <f t="shared" ca="1" si="2"/>
@@ -2023,27 +2024,27 @@
       </c>
       <c r="D29">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G29">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H29">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J29">
         <f t="shared" ca="1" si="4"/>
@@ -2051,7 +2052,7 @@
       </c>
       <c r="K29">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L29">
         <f t="shared" ca="1" si="4"/>
@@ -2059,21 +2060,21 @@
       </c>
       <c r="M29">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N29">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="B30">
         <f t="shared" ca="1" si="1"/>
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="C30">
         <f t="shared" ca="1" si="2"/>
@@ -2081,11 +2082,11 @@
       </c>
       <c r="D30">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30">
         <f t="shared" ca="1" si="4"/>
@@ -2097,27 +2098,27 @@
       </c>
       <c r="H30">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I30">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J30">
         <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K30">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L30">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M30">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N30">
         <f t="shared" ca="1" si="4"/>
@@ -2127,11 +2128,11 @@
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="B31">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="C31">
         <f t="shared" ca="1" si="2"/>
@@ -2139,31 +2140,31 @@
       </c>
       <c r="D31">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31">
         <f t="shared" ca="1" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G31">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H31">
         <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I31">
         <f t="shared" ref="I31:N31" ca="1" si="5">RANDBETWEEN(1, 5)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K31">
         <f t="shared" ca="1" si="5"/>
@@ -2171,15 +2172,70 @@
       </c>
       <c r="L31">
         <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M31">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N31">
         <f t="shared" ca="1" si="5"/>
-        <v>3</v>
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD886EC-0CCF-41AE-98FD-302CB1DC3A83}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>